<commit_message>
Populate Market - Demand-Side Scan with real Cedar Crest sales data
Filter source workbook's Summary tab to customers with Weeks Ordered >= 3,
then use that base to drive four panels:

- Overall Market Penetration by Distance: descending-by-distance bar chart,
  even 50-mile bands, real counts/percentages.
- Customer Cases by Distance: per-customer scatter (cases, since revenue
  isn't tracked), name-derived category legend with click-to-toggle,
  log-scale y-axis, top 3 outlier accounts excluded and noted.
- Case Volume by Channel (renamed from Demand Growth by Channel): total
  cases per category, replacing placeholder YoY figures.
- Demand Indicators by Segment: real category rows with % of Orders in
  place of YoY Growth.

Penetration by Range & Customer Type left as pending placeholder per request.
Adds backing data files for the new/changed panels and the filtered source
workbook itself.
</commit_message>
<xml_diff>
--- a/data/Demand Indicators by Segment.xlsx
+++ b/data/Demand Indicators by Segment.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +29,14 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +59,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,14 +432,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,7 +455,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>YoY Growth %</t>
+          <t>% of Orders</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -455,41 +470,191 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Convenience Store / Gas</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Route density -- largest customer count (557) and highest order frequency (~33 orders/yr avg)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Maintain</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Farms, churches, campgrounds, and 3 large wholesale/distributor accounts</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Defend</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Supermarket / Grocery</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Large-format accounts -- fewest locations (110) but highest cases per account</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ice Cream / Dessert Shop</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Seasonal scoop-shop demand, longest average haul (105 mi)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>School / Institutional</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Direct-to-Consumer</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Local/Premium Retail</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Category Average</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Distributor / Wholesale</t>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Academic-calendar driven, K-12 milk program contracts</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Invest</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Coffee Shop</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>High-frequency, small-batch reorders (Biggby, Scooters, independents)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Maintain</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Restaurant / Food Service</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Smallest, most dispersed segment (avg 112 mi) -- lowest order share</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Source: Cedar Crest Weekly Sales Database - April2025-March2026.xlsx, 'Summary - All Weeks' tab, customers with Weeks Ordered &gt;= 3 (1,523 of 1,730 customers; 37,496 order-rows). % of Orders = each category's share of total order-rows (one row = one customer's order in one week). Same name-based categories as 'Customer Cases by Distance' and 'Case Volume by Channel' (directional, not an exact type field). Demand Level is derived from % of Orders (&gt;=20% High, 5-20% Moderate, &lt;5% Low). Primary Driver and Recommended Posture are qualitative judgment calls grounded in order share, case volume, and average distance -- not separately sourced metrics.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A10:E10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>